<commit_message>
docs: PRIVACY.md gizlilik politikasi eklendi (TR/EN)
</commit_message>
<xml_diff>
--- a/OSSRequestForm-v4.xlsx
+++ b/OSSRequestForm-v4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hzk\source\repos\MikroUpdate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0253E485-FA97-4FFD-BABB-B7259E80EABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38110D0E-BB25-4A72-BA59-14B67440569D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3BFD8953-F348-4C25-9E04-BE37B4BD5AA3}"/>
   </bookViews>
@@ -699,10 +699,10 @@
     <t>Huseyin Kucuk</t>
   </si>
   <si>
-    <t>This program will not transfer any information to other networked systems unless specifically requested by the user or the person installing or operating it.</t>
-  </si>
-  <si>
     <t>MikroUpdate is actively maintained with regular releases (v1.19.2 as of July 2025). GitHub repository: https://github.com/hzkucuk/MikroUpdate - Public repository with full source code, documentation (README, CHANGELOG, FEATURES), automated CI/CD via GitHub Actions, and multiple releases with installer artifacts.</t>
+  </si>
+  <si>
+    <t>https://github.com/hzkucuk/MikroUpdate/blob/master/PRIVACY.md</t>
   </si>
 </sst>
 </file>
@@ -889,17 +889,17 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1303,7 +1303,7 @@
         <v>55</v>
       </c>
       <c r="E2" s="8"/>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="24" t="s">
         <v>32</v>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
         <v>55</v>
       </c>
       <c r="E4" s="8"/>
-      <c r="F4" s="21" t="s">
+      <c r="F4" s="24" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1349,14 +1349,14 @@
         <v>29</v>
       </c>
       <c r="E6" s="8"/>
-      <c r="F6" s="21" t="s">
+      <c r="F6" s="24" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4"/>
       <c r="E7" s="8"/>
-      <c r="F7" s="21"/>
+      <c r="F7" s="24"/>
     </row>
     <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
@@ -1372,7 +1372,7 @@
         <v>56</v>
       </c>
       <c r="E8" s="8"/>
-      <c r="F8" s="21" t="s">
+      <c r="F8" s="24" t="s">
         <v>37</v>
       </c>
       <c r="I8" s="9"/>
@@ -1397,7 +1397,7 @@
         <v>57</v>
       </c>
       <c r="E10" s="8"/>
-      <c r="F10" s="21" t="s">
+      <c r="F10" s="24" t="s">
         <v>34</v>
       </c>
       <c r="I10" s="7"/>
@@ -1422,7 +1422,7 @@
         <v>57</v>
       </c>
       <c r="E12" s="8"/>
-      <c r="F12" s="21" t="s">
+      <c r="F12" s="24" t="s">
         <v>39</v>
       </c>
     </row>
@@ -1443,7 +1443,7 @@
         <v>58</v>
       </c>
       <c r="E14" s="8"/>
-      <c r="F14" s="21" t="s">
+      <c r="F14" s="24" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1452,7 +1452,7 @@
       <c r="E15" s="8"/>
       <c r="F15" s="22"/>
     </row>
-    <row r="16" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="4"/>
       <c r="B16" s="11" t="s">
         <v>11</v>
@@ -1461,10 +1461,10 @@
         <v>19</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E16" s="8"/>
-      <c r="F16" s="21" t="s">
+      <c r="F16" s="24" t="s">
         <v>36</v>
       </c>
     </row>
@@ -1483,7 +1483,7 @@
       </c>
       <c r="D18" s="16"/>
       <c r="E18" s="8"/>
-      <c r="F18" s="21" t="s">
+      <c r="F18" s="24" t="s">
         <v>35</v>
       </c>
     </row>
@@ -1506,7 +1506,7 @@
         <v>59</v>
       </c>
       <c r="E20" s="8"/>
-      <c r="F20" s="21" t="s">
+      <c r="F20" s="24" t="s">
         <v>38</v>
       </c>
     </row>
@@ -1549,17 +1549,17 @@
         <v>15</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E24" s="12"/>
-      <c r="F24" s="24" t="s">
+      <c r="F24" s="23" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="4"/>
       <c r="E25" s="8"/>
-      <c r="F25" s="24"/>
+      <c r="F25" s="23"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
@@ -1575,7 +1575,7 @@
         <v>61</v>
       </c>
       <c r="E26" s="8"/>
-      <c r="F26" s="23" t="s">
+      <c r="F26" s="21" t="s">
         <v>45</v>
       </c>
     </row>
@@ -1598,7 +1598,7 @@
         <v>53</v>
       </c>
       <c r="E28" s="8"/>
-      <c r="F28" s="23" t="s">
+      <c r="F28" s="21" t="s">
         <v>46</v>
       </c>
     </row>
@@ -1618,7 +1618,7 @@
         <v>52</v>
       </c>
       <c r="E30" s="8"/>
-      <c r="F30" s="23" t="s">
+      <c r="F30" s="21" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1648,11 +1648,6 @@
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="14">
-    <mergeCell ref="F30:F31"/>
-    <mergeCell ref="F26:F27"/>
-    <mergeCell ref="F28:F29"/>
-    <mergeCell ref="F24:F25"/>
-    <mergeCell ref="F6:F7"/>
     <mergeCell ref="F2:F3"/>
     <mergeCell ref="F4:F5"/>
     <mergeCell ref="F20:F21"/>
@@ -1662,6 +1657,11 @@
     <mergeCell ref="F18:F19"/>
     <mergeCell ref="F16:F17"/>
     <mergeCell ref="F8:F9"/>
+    <mergeCell ref="F30:F31"/>
+    <mergeCell ref="F26:F27"/>
+    <mergeCell ref="F28:F29"/>
+    <mergeCell ref="F24:F25"/>
+    <mergeCell ref="F6:F7"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation showInputMessage="1" showErrorMessage="1" sqref="D7" xr:uid="{164A41B7-150B-40BD-8525-8D11720296A6}"/>

</xml_diff>